<commit_message>
Improve README quility and extend it
</commit_message>
<xml_diff>
--- a/verify/vPlan/block/lsu.xlsx
+++ b/verify/vPlan/block/lsu.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="18">
   <si>
     <t xml:space="preserve">Requirement Location</t>
   </si>
@@ -58,7 +58,25 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
+    <t xml:space="preserve">Store</t>
+  </si>
+  <si>
     <t xml:space="preserve">not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misaligned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stalling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Err-Answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interrupt</t>
   </si>
 </sst>
 </file>
@@ -73,6 +91,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -132,16 +151,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -164,7 +199,6 @@
           <bgColor rgb="FFCCFFCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -175,7 +209,6 @@
           <bgColor rgb="FFFFFFCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -186,7 +219,6 @@
           <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -366,1647 +398,2148 @@
   <dimension ref="A1:O514"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="25.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="23.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="5" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K6" s="1" t="s">
-        <v>11</v>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="4"/>
+      <c r="K6" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K7" s="1" t="s">
-        <v>11</v>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K8" s="1" t="s">
-        <v>11</v>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K9" s="1" t="s">
-        <v>11</v>
+      <c r="B9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K10" s="1" t="s">
-        <v>11</v>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K11" s="1" t="s">
-        <v>11</v>
+      <c r="B11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K12" s="1" t="s">
-        <v>11</v>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K13" s="1" t="s">
-        <v>11</v>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K14" s="1" t="s">
-        <v>11</v>
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K15" s="1" t="s">
-        <v>11</v>
+      <c r="B15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K16" s="1" t="s">
-        <v>11</v>
+      <c r="B16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K17" s="1" t="s">
-        <v>11</v>
+      <c r="B17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K18" s="1" t="s">
-        <v>11</v>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K19" s="1" t="s">
-        <v>11</v>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K20" s="1" t="s">
-        <v>11</v>
+      <c r="B20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K21" s="1" t="s">
-        <v>11</v>
+      <c r="B21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K22" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K23" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K24" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K25" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K26" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K27" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K28" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="O28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="5"/>
+      <c r="O28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K29" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K30" s="1"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K31" s="1"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K32" s="1"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K33" s="1"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K34" s="1"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K35" s="1"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K36" s="1"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K37" s="1"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K38" s="1"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K39" s="1"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K40" s="1"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K41" s="1"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K42" s="1"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K43" s="1"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K44" s="1"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K45" s="1"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K46" s="1"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K47" s="1"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="4"/>
+      <c r="K47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K48" s="1"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K49" s="1"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K50" s="1"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K51" s="1"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K52" s="1"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K53" s="1"/>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="4"/>
+      <c r="K53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K54" s="1"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="2"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K55" s="1"/>
+      <c r="K55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K56" s="1"/>
+      <c r="K56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K57" s="1"/>
+      <c r="K57" s="5"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K58" s="1"/>
+      <c r="K58" s="5"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K59" s="1"/>
+      <c r="K59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K60" s="1"/>
+      <c r="K60" s="5"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K61" s="1"/>
+      <c r="K61" s="5"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K62" s="1"/>
+      <c r="K62" s="5"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K63" s="1"/>
+      <c r="K63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K64" s="1"/>
+      <c r="K64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K65" s="1"/>
+      <c r="K65" s="5"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K66" s="1"/>
+      <c r="K66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K67" s="1"/>
+      <c r="K67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K68" s="1"/>
+      <c r="K68" s="5"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K69" s="1"/>
+      <c r="K69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K70" s="1"/>
+      <c r="K70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K71" s="1"/>
+      <c r="K71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K72" s="1"/>
+      <c r="K72" s="5"/>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K73" s="1"/>
+      <c r="K73" s="5"/>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K74" s="1"/>
+      <c r="K74" s="5"/>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K75" s="1"/>
+      <c r="K75" s="5"/>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K76" s="1"/>
+      <c r="K76" s="5"/>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K77" s="1"/>
+      <c r="K77" s="5"/>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K78" s="1"/>
+      <c r="K78" s="5"/>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K79" s="1"/>
+      <c r="K79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K80" s="1"/>
+      <c r="K80" s="5"/>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K81" s="1"/>
+      <c r="K81" s="5"/>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K82" s="1"/>
+      <c r="K82" s="5"/>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K83" s="1"/>
+      <c r="K83" s="5"/>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K84" s="1"/>
+      <c r="K84" s="5"/>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K85" s="1"/>
+      <c r="K85" s="5"/>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K86" s="1"/>
+      <c r="K86" s="5"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K87" s="1"/>
+      <c r="K87" s="5"/>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K88" s="1"/>
+      <c r="K88" s="5"/>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K89" s="1"/>
+      <c r="K89" s="5"/>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K90" s="1"/>
+      <c r="K90" s="5"/>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K91" s="1"/>
+      <c r="K91" s="5"/>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K92" s="1"/>
+      <c r="K92" s="5"/>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K93" s="1"/>
+      <c r="K93" s="5"/>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K94" s="1"/>
+      <c r="K94" s="5"/>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K95" s="1"/>
+      <c r="K95" s="5"/>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K96" s="1"/>
+      <c r="K96" s="5"/>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K97" s="1"/>
+      <c r="K97" s="5"/>
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K98" s="1"/>
+      <c r="K98" s="5"/>
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K99" s="1"/>
+      <c r="K99" s="5"/>
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K100" s="1"/>
+      <c r="K100" s="5"/>
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K101" s="1"/>
+      <c r="K101" s="5"/>
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K102" s="1"/>
+      <c r="K102" s="5"/>
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K103" s="1"/>
+      <c r="K103" s="5"/>
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K104" s="1"/>
+      <c r="K104" s="5"/>
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K105" s="1"/>
+      <c r="K105" s="5"/>
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K106" s="1"/>
+      <c r="K106" s="5"/>
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K107" s="1"/>
+      <c r="K107" s="5"/>
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K108" s="1"/>
+      <c r="K108" s="5"/>
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K109" s="1"/>
+      <c r="K109" s="5"/>
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K110" s="1"/>
+      <c r="K110" s="5"/>
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K111" s="1"/>
+      <c r="K111" s="5"/>
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K112" s="1"/>
+      <c r="K112" s="5"/>
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K113" s="1"/>
+      <c r="K113" s="5"/>
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K114" s="1"/>
+      <c r="K114" s="5"/>
     </row>
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K115" s="1"/>
+      <c r="K115" s="5"/>
     </row>
     <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K116" s="1"/>
+      <c r="K116" s="5"/>
     </row>
     <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K117" s="1"/>
+      <c r="K117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K118" s="1"/>
+      <c r="K118" s="5"/>
     </row>
     <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K119" s="1"/>
+      <c r="K119" s="5"/>
     </row>
     <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K120" s="1"/>
+      <c r="K120" s="5"/>
     </row>
     <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K121" s="1"/>
+      <c r="K121" s="5"/>
     </row>
     <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K122" s="1"/>
+      <c r="K122" s="5"/>
     </row>
     <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K123" s="1"/>
+      <c r="K123" s="5"/>
     </row>
     <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K124" s="1"/>
+      <c r="K124" s="5"/>
     </row>
     <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K125" s="1"/>
+      <c r="K125" s="5"/>
     </row>
     <row r="126" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K126" s="1"/>
+      <c r="K126" s="5"/>
     </row>
     <row r="127" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K127" s="1"/>
+      <c r="K127" s="5"/>
     </row>
     <row r="128" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K128" s="1"/>
+      <c r="K128" s="5"/>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K129" s="1"/>
+      <c r="K129" s="5"/>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K130" s="1"/>
+      <c r="K130" s="5"/>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K131" s="1"/>
+      <c r="K131" s="5"/>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K132" s="1"/>
+      <c r="K132" s="5"/>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K133" s="1"/>
+      <c r="K133" s="5"/>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K134" s="1"/>
+      <c r="K134" s="5"/>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K135" s="1"/>
+      <c r="K135" s="5"/>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K136" s="1"/>
+      <c r="K136" s="5"/>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K137" s="1"/>
+      <c r="K137" s="5"/>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K138" s="1"/>
+      <c r="K138" s="5"/>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K139" s="1"/>
+      <c r="K139" s="5"/>
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K140" s="1"/>
+      <c r="K140" s="5"/>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K141" s="1"/>
+      <c r="K141" s="5"/>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K142" s="1"/>
+      <c r="K142" s="5"/>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K143" s="1"/>
+      <c r="K143" s="5"/>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K144" s="1"/>
+      <c r="K144" s="5"/>
     </row>
     <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K145" s="1"/>
+      <c r="K145" s="5"/>
     </row>
     <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K146" s="1"/>
+      <c r="K146" s="5"/>
     </row>
     <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K147" s="1"/>
+      <c r="K147" s="5"/>
     </row>
     <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K148" s="1"/>
+      <c r="K148" s="5"/>
     </row>
     <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K149" s="1"/>
+      <c r="K149" s="5"/>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K150" s="1"/>
+      <c r="K150" s="5"/>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K151" s="1"/>
+      <c r="K151" s="5"/>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K152" s="1"/>
+      <c r="K152" s="5"/>
     </row>
     <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K153" s="1"/>
+      <c r="K153" s="5"/>
     </row>
     <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K154" s="1"/>
+      <c r="K154" s="5"/>
     </row>
     <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K155" s="1"/>
+      <c r="K155" s="5"/>
     </row>
     <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K156" s="1"/>
+      <c r="K156" s="5"/>
     </row>
     <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K157" s="1"/>
+      <c r="K157" s="5"/>
     </row>
     <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K158" s="1"/>
+      <c r="K158" s="5"/>
     </row>
     <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K159" s="1"/>
+      <c r="K159" s="5"/>
     </row>
     <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K160" s="1"/>
+      <c r="K160" s="5"/>
     </row>
     <row r="161" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K161" s="1"/>
+      <c r="K161" s="5"/>
     </row>
     <row r="162" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K162" s="1"/>
+      <c r="K162" s="5"/>
     </row>
     <row r="163" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K163" s="1"/>
+      <c r="K163" s="5"/>
     </row>
     <row r="164" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K164" s="1"/>
+      <c r="K164" s="5"/>
     </row>
     <row r="165" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K165" s="1"/>
+      <c r="K165" s="5"/>
     </row>
     <row r="166" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K166" s="1"/>
+      <c r="K166" s="5"/>
     </row>
     <row r="167" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K167" s="1"/>
+      <c r="K167" s="5"/>
     </row>
     <row r="168" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K168" s="1"/>
+      <c r="K168" s="5"/>
     </row>
     <row r="169" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K169" s="1"/>
+      <c r="K169" s="5"/>
     </row>
     <row r="170" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K170" s="1"/>
+      <c r="K170" s="5"/>
     </row>
     <row r="171" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K171" s="1"/>
+      <c r="K171" s="5"/>
     </row>
     <row r="172" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K172" s="1"/>
+      <c r="K172" s="5"/>
     </row>
     <row r="173" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K173" s="1"/>
+      <c r="K173" s="5"/>
     </row>
     <row r="174" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K174" s="1"/>
+      <c r="K174" s="5"/>
     </row>
     <row r="175" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K175" s="1"/>
+      <c r="K175" s="5"/>
     </row>
     <row r="176" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K176" s="1"/>
+      <c r="K176" s="5"/>
     </row>
     <row r="177" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K177" s="1"/>
+      <c r="K177" s="5"/>
     </row>
     <row r="178" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K178" s="1"/>
+      <c r="K178" s="5"/>
     </row>
     <row r="179" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K179" s="1"/>
+      <c r="K179" s="5"/>
     </row>
     <row r="180" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K180" s="1"/>
+      <c r="K180" s="5"/>
     </row>
     <row r="181" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K181" s="1"/>
+      <c r="K181" s="5"/>
     </row>
     <row r="182" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K182" s="1"/>
+      <c r="K182" s="5"/>
     </row>
     <row r="183" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K183" s="1"/>
+      <c r="K183" s="5"/>
     </row>
     <row r="184" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K184" s="1"/>
+      <c r="K184" s="5"/>
     </row>
     <row r="185" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K185" s="1"/>
+      <c r="K185" s="5"/>
     </row>
     <row r="186" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K186" s="1"/>
+      <c r="K186" s="5"/>
     </row>
     <row r="187" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K187" s="1"/>
+      <c r="K187" s="5"/>
     </row>
     <row r="188" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K188" s="1"/>
+      <c r="K188" s="5"/>
     </row>
     <row r="189" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K189" s="1"/>
+      <c r="K189" s="5"/>
     </row>
     <row r="190" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K190" s="1"/>
+      <c r="K190" s="5"/>
     </row>
     <row r="191" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K191" s="1"/>
+      <c r="K191" s="5"/>
     </row>
     <row r="192" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K192" s="1"/>
+      <c r="K192" s="5"/>
     </row>
     <row r="193" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K193" s="1"/>
+      <c r="K193" s="5"/>
     </row>
     <row r="194" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K194" s="1"/>
+      <c r="K194" s="5"/>
     </row>
     <row r="195" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K195" s="1"/>
+      <c r="K195" s="5"/>
     </row>
     <row r="196" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K196" s="1"/>
+      <c r="K196" s="5"/>
     </row>
     <row r="197" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K197" s="1"/>
+      <c r="K197" s="5"/>
     </row>
     <row r="198" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K198" s="1"/>
+      <c r="K198" s="5"/>
     </row>
     <row r="199" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K199" s="1"/>
+      <c r="K199" s="5"/>
     </row>
     <row r="200" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K200" s="1"/>
+      <c r="K200" s="5"/>
     </row>
     <row r="201" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K201" s="1"/>
+      <c r="K201" s="5"/>
     </row>
     <row r="202" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K202" s="1"/>
+      <c r="K202" s="5"/>
     </row>
     <row r="203" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K203" s="1"/>
+      <c r="K203" s="5"/>
     </row>
     <row r="204" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K204" s="1"/>
+      <c r="K204" s="5"/>
     </row>
     <row r="205" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K205" s="1"/>
+      <c r="K205" s="5"/>
     </row>
     <row r="206" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K206" s="1"/>
+      <c r="K206" s="5"/>
     </row>
     <row r="207" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K207" s="1"/>
+      <c r="K207" s="5"/>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K208" s="1"/>
+      <c r="K208" s="5"/>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K209" s="1"/>
+      <c r="K209" s="5"/>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K210" s="1"/>
+      <c r="K210" s="5"/>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K211" s="1"/>
+      <c r="K211" s="5"/>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K212" s="1"/>
+      <c r="K212" s="5"/>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K213" s="1"/>
+      <c r="K213" s="5"/>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K214" s="1"/>
+      <c r="K214" s="5"/>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K215" s="1"/>
+      <c r="K215" s="5"/>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K216" s="1"/>
+      <c r="K216" s="5"/>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K217" s="1"/>
+      <c r="K217" s="5"/>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K218" s="1"/>
+      <c r="K218" s="5"/>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K219" s="1"/>
+      <c r="K219" s="5"/>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K220" s="1"/>
+      <c r="K220" s="5"/>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K221" s="1"/>
+      <c r="K221" s="5"/>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K222" s="1"/>
+      <c r="K222" s="5"/>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K223" s="1"/>
+      <c r="K223" s="5"/>
     </row>
     <row r="224" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K224" s="1"/>
+      <c r="K224" s="5"/>
     </row>
     <row r="225" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K225" s="1"/>
+      <c r="K225" s="5"/>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K226" s="1"/>
+      <c r="K226" s="5"/>
     </row>
     <row r="227" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K227" s="1"/>
+      <c r="K227" s="5"/>
     </row>
     <row r="228" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K228" s="1"/>
+      <c r="K228" s="5"/>
     </row>
     <row r="229" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K229" s="1"/>
+      <c r="K229" s="5"/>
     </row>
     <row r="230" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K230" s="1"/>
+      <c r="K230" s="5"/>
     </row>
     <row r="231" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K231" s="1"/>
+      <c r="K231" s="5"/>
     </row>
     <row r="232" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K232" s="1"/>
+      <c r="K232" s="5"/>
     </row>
     <row r="233" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K233" s="1"/>
+      <c r="K233" s="5"/>
     </row>
     <row r="234" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K234" s="1"/>
+      <c r="K234" s="5"/>
     </row>
     <row r="235" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K235" s="1"/>
+      <c r="K235" s="5"/>
     </row>
     <row r="236" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K236" s="1"/>
+      <c r="K236" s="5"/>
     </row>
     <row r="237" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K237" s="1"/>
+      <c r="K237" s="5"/>
     </row>
     <row r="238" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K238" s="1"/>
+      <c r="K238" s="5"/>
     </row>
     <row r="239" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K239" s="1"/>
+      <c r="K239" s="5"/>
     </row>
     <row r="240" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K240" s="1"/>
+      <c r="K240" s="5"/>
     </row>
     <row r="241" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K241" s="1"/>
+      <c r="K241" s="5"/>
     </row>
     <row r="242" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K242" s="1"/>
+      <c r="K242" s="5"/>
     </row>
     <row r="243" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K243" s="1"/>
+      <c r="K243" s="5"/>
     </row>
     <row r="244" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K244" s="1"/>
+      <c r="K244" s="5"/>
     </row>
     <row r="245" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K245" s="1"/>
+      <c r="K245" s="5"/>
     </row>
     <row r="246" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K246" s="1"/>
+      <c r="K246" s="5"/>
     </row>
     <row r="247" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K247" s="1"/>
+      <c r="K247" s="5"/>
     </row>
     <row r="248" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K248" s="1"/>
+      <c r="K248" s="5"/>
     </row>
     <row r="249" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K249" s="1"/>
+      <c r="K249" s="5"/>
     </row>
     <row r="250" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K250" s="1"/>
+      <c r="K250" s="5"/>
     </row>
     <row r="251" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K251" s="1"/>
+      <c r="K251" s="5"/>
     </row>
     <row r="252" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K252" s="1"/>
+      <c r="K252" s="5"/>
     </row>
     <row r="253" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K253" s="1"/>
+      <c r="K253" s="5"/>
     </row>
     <row r="254" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K254" s="1"/>
+      <c r="K254" s="5"/>
     </row>
     <row r="255" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K255" s="1"/>
+      <c r="K255" s="5"/>
     </row>
     <row r="256" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K256" s="1"/>
+      <c r="K256" s="5"/>
     </row>
     <row r="257" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K257" s="1"/>
+      <c r="K257" s="5"/>
     </row>
     <row r="258" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K258" s="1"/>
+      <c r="K258" s="5"/>
     </row>
     <row r="259" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K259" s="1"/>
+      <c r="K259" s="5"/>
     </row>
     <row r="260" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K260" s="1"/>
+      <c r="K260" s="5"/>
     </row>
     <row r="261" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K261" s="1"/>
+      <c r="K261" s="5"/>
     </row>
     <row r="262" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K262" s="1"/>
+      <c r="K262" s="5"/>
     </row>
     <row r="263" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K263" s="1"/>
+      <c r="K263" s="5"/>
     </row>
     <row r="264" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K264" s="1"/>
+      <c r="K264" s="5"/>
     </row>
     <row r="265" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K265" s="1"/>
+      <c r="K265" s="5"/>
     </row>
     <row r="266" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K266" s="1"/>
+      <c r="K266" s="5"/>
     </row>
     <row r="267" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K267" s="1"/>
+      <c r="K267" s="5"/>
     </row>
     <row r="268" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K268" s="1"/>
+      <c r="K268" s="5"/>
     </row>
     <row r="269" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K269" s="1"/>
+      <c r="K269" s="5"/>
     </row>
     <row r="270" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K270" s="1"/>
+      <c r="K270" s="5"/>
     </row>
     <row r="271" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K271" s="1"/>
+      <c r="K271" s="5"/>
     </row>
     <row r="272" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K272" s="1"/>
+      <c r="K272" s="5"/>
     </row>
     <row r="273" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K273" s="1"/>
+      <c r="K273" s="5"/>
     </row>
     <row r="274" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K274" s="1"/>
+      <c r="K274" s="5"/>
     </row>
     <row r="275" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K275" s="1"/>
+      <c r="K275" s="5"/>
     </row>
     <row r="276" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K276" s="1"/>
+      <c r="K276" s="5"/>
     </row>
     <row r="277" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K277" s="1"/>
+      <c r="K277" s="5"/>
     </row>
     <row r="278" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K278" s="1"/>
+      <c r="K278" s="5"/>
     </row>
     <row r="279" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K279" s="1"/>
+      <c r="K279" s="5"/>
     </row>
     <row r="280" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K280" s="1"/>
+      <c r="K280" s="5"/>
     </row>
     <row r="281" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K281" s="1"/>
+      <c r="K281" s="5"/>
     </row>
     <row r="282" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K282" s="1"/>
+      <c r="K282" s="5"/>
     </row>
     <row r="283" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K283" s="1"/>
+      <c r="K283" s="5"/>
     </row>
     <row r="284" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K284" s="1"/>
+      <c r="K284" s="5"/>
     </row>
     <row r="285" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K285" s="1"/>
+      <c r="K285" s="5"/>
     </row>
     <row r="286" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K286" s="1"/>
+      <c r="K286" s="5"/>
     </row>
     <row r="287" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K287" s="1"/>
+      <c r="K287" s="5"/>
     </row>
     <row r="288" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K288" s="1"/>
+      <c r="K288" s="5"/>
     </row>
     <row r="289" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K289" s="1"/>
+      <c r="K289" s="5"/>
     </row>
     <row r="290" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K290" s="1"/>
+      <c r="K290" s="5"/>
     </row>
     <row r="291" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K291" s="1"/>
+      <c r="K291" s="5"/>
     </row>
     <row r="292" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K292" s="1"/>
+      <c r="K292" s="5"/>
     </row>
     <row r="293" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K293" s="1"/>
+      <c r="K293" s="5"/>
     </row>
     <row r="294" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K294" s="1"/>
+      <c r="K294" s="5"/>
     </row>
     <row r="295" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K295" s="1"/>
+      <c r="K295" s="5"/>
     </row>
     <row r="296" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K296" s="1"/>
+      <c r="K296" s="5"/>
     </row>
     <row r="297" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K297" s="1"/>
+      <c r="K297" s="5"/>
     </row>
     <row r="298" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K298" s="1"/>
+      <c r="K298" s="5"/>
     </row>
     <row r="299" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K299" s="1"/>
+      <c r="K299" s="5"/>
     </row>
     <row r="300" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K300" s="1"/>
+      <c r="K300" s="5"/>
     </row>
     <row r="301" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K301" s="1"/>
+      <c r="K301" s="5"/>
     </row>
     <row r="302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K302" s="1"/>
+      <c r="K302" s="5"/>
     </row>
     <row r="303" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K303" s="1"/>
+      <c r="K303" s="5"/>
     </row>
     <row r="304" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K304" s="1"/>
+      <c r="K304" s="5"/>
     </row>
     <row r="305" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K305" s="1"/>
+      <c r="K305" s="5"/>
     </row>
     <row r="306" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K306" s="1"/>
+      <c r="K306" s="5"/>
     </row>
     <row r="307" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K307" s="1"/>
+      <c r="K307" s="5"/>
     </row>
     <row r="308" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K308" s="1"/>
+      <c r="K308" s="5"/>
     </row>
     <row r="309" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K309" s="1"/>
+      <c r="K309" s="5"/>
     </row>
     <row r="310" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K310" s="1"/>
+      <c r="K310" s="5"/>
     </row>
     <row r="311" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K311" s="1"/>
+      <c r="K311" s="5"/>
     </row>
     <row r="312" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K312" s="1"/>
+      <c r="K312" s="5"/>
     </row>
     <row r="313" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K313" s="1"/>
+      <c r="K313" s="5"/>
     </row>
     <row r="314" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K314" s="1"/>
+      <c r="K314" s="5"/>
     </row>
     <row r="315" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K315" s="1"/>
+      <c r="K315" s="5"/>
     </row>
     <row r="316" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K316" s="1"/>
+      <c r="K316" s="5"/>
     </row>
     <row r="317" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K317" s="1"/>
+      <c r="K317" s="5"/>
     </row>
     <row r="318" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K318" s="1"/>
+      <c r="K318" s="5"/>
     </row>
     <row r="319" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K319" s="1"/>
+      <c r="K319" s="5"/>
     </row>
     <row r="320" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K320" s="1"/>
+      <c r="K320" s="5"/>
     </row>
     <row r="321" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K321" s="1"/>
+      <c r="K321" s="5"/>
     </row>
     <row r="322" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K322" s="1"/>
+      <c r="K322" s="5"/>
     </row>
     <row r="323" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K323" s="1"/>
+      <c r="K323" s="5"/>
     </row>
     <row r="324" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K324" s="1"/>
+      <c r="K324" s="5"/>
     </row>
     <row r="325" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K325" s="1"/>
+      <c r="K325" s="5"/>
     </row>
     <row r="326" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K326" s="1"/>
+      <c r="K326" s="5"/>
     </row>
     <row r="327" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K327" s="1"/>
+      <c r="K327" s="5"/>
     </row>
     <row r="328" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K328" s="1"/>
+      <c r="K328" s="5"/>
     </row>
     <row r="329" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K329" s="1"/>
+      <c r="K329" s="5"/>
     </row>
     <row r="330" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K330" s="1"/>
+      <c r="K330" s="5"/>
     </row>
     <row r="331" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K331" s="1"/>
+      <c r="K331" s="5"/>
     </row>
     <row r="332" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K332" s="1"/>
+      <c r="K332" s="5"/>
     </row>
     <row r="333" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K333" s="1"/>
+      <c r="K333" s="5"/>
     </row>
     <row r="334" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K334" s="1"/>
+      <c r="K334" s="5"/>
     </row>
     <row r="335" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K335" s="1"/>
+      <c r="K335" s="5"/>
     </row>
     <row r="336" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K336" s="1"/>
+      <c r="K336" s="5"/>
     </row>
     <row r="337" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K337" s="1"/>
+      <c r="K337" s="5"/>
     </row>
     <row r="338" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K338" s="1"/>
+      <c r="K338" s="5"/>
     </row>
     <row r="339" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K339" s="1"/>
+      <c r="K339" s="5"/>
     </row>
     <row r="340" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K340" s="1"/>
+      <c r="K340" s="5"/>
     </row>
     <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K341" s="1"/>
+      <c r="K341" s="5"/>
     </row>
     <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K342" s="1"/>
+      <c r="K342" s="5"/>
     </row>
     <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K343" s="1"/>
+      <c r="K343" s="5"/>
     </row>
     <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K344" s="1"/>
+      <c r="K344" s="5"/>
     </row>
     <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K345" s="1"/>
+      <c r="K345" s="5"/>
     </row>
     <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K346" s="1"/>
+      <c r="K346" s="5"/>
     </row>
     <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K347" s="1"/>
+      <c r="K347" s="5"/>
     </row>
     <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K348" s="1"/>
+      <c r="K348" s="5"/>
     </row>
     <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K349" s="1"/>
+      <c r="K349" s="5"/>
     </row>
     <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K350" s="1"/>
+      <c r="K350" s="5"/>
     </row>
     <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K351" s="1"/>
+      <c r="K351" s="5"/>
     </row>
     <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K352" s="1"/>
+      <c r="K352" s="5"/>
     </row>
     <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K353" s="1"/>
+      <c r="K353" s="5"/>
     </row>
     <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K354" s="1"/>
+      <c r="K354" s="5"/>
     </row>
     <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K355" s="1"/>
+      <c r="K355" s="5"/>
     </row>
     <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K356" s="1"/>
+      <c r="K356" s="5"/>
     </row>
     <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K357" s="1"/>
+      <c r="K357" s="5"/>
     </row>
     <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K358" s="1"/>
+      <c r="K358" s="5"/>
     </row>
     <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K359" s="1"/>
+      <c r="K359" s="5"/>
     </row>
     <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K360" s="1"/>
+      <c r="K360" s="5"/>
     </row>
     <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K361" s="1"/>
+      <c r="K361" s="5"/>
     </row>
     <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K362" s="1"/>
+      <c r="K362" s="5"/>
     </row>
     <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K363" s="1"/>
+      <c r="K363" s="5"/>
     </row>
     <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K364" s="1"/>
+      <c r="K364" s="5"/>
     </row>
     <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K365" s="1"/>
+      <c r="K365" s="5"/>
     </row>
     <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K366" s="1"/>
+      <c r="K366" s="5"/>
     </row>
     <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K367" s="1"/>
+      <c r="K367" s="5"/>
     </row>
     <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K368" s="1"/>
+      <c r="K368" s="5"/>
     </row>
     <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K369" s="1"/>
+      <c r="K369" s="5"/>
     </row>
     <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K370" s="1"/>
+      <c r="K370" s="5"/>
     </row>
     <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K371" s="1"/>
+      <c r="K371" s="5"/>
     </row>
     <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K372" s="1"/>
+      <c r="K372" s="5"/>
     </row>
     <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K373" s="1"/>
+      <c r="K373" s="5"/>
     </row>
     <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K374" s="1"/>
+      <c r="K374" s="5"/>
     </row>
     <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K375" s="1"/>
+      <c r="K375" s="5"/>
     </row>
     <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K376" s="1"/>
+      <c r="K376" s="5"/>
     </row>
     <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K377" s="1"/>
+      <c r="K377" s="5"/>
     </row>
     <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K378" s="1"/>
+      <c r="K378" s="5"/>
     </row>
     <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K379" s="1"/>
+      <c r="K379" s="5"/>
     </row>
     <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K380" s="1"/>
+      <c r="K380" s="5"/>
     </row>
     <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K381" s="1"/>
+      <c r="K381" s="5"/>
     </row>
     <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K382" s="1"/>
+      <c r="K382" s="5"/>
     </row>
     <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K383" s="1"/>
+      <c r="K383" s="5"/>
     </row>
     <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K384" s="1"/>
+      <c r="K384" s="5"/>
     </row>
     <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K385" s="1"/>
+      <c r="K385" s="5"/>
     </row>
     <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K386" s="1"/>
+      <c r="K386" s="5"/>
     </row>
     <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K387" s="1"/>
+      <c r="K387" s="5"/>
     </row>
     <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K388" s="1"/>
+      <c r="K388" s="5"/>
     </row>
     <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K389" s="1"/>
+      <c r="K389" s="5"/>
     </row>
     <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K390" s="1"/>
+      <c r="K390" s="5"/>
     </row>
     <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K391" s="1"/>
+      <c r="K391" s="5"/>
     </row>
     <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K392" s="1"/>
+      <c r="K392" s="5"/>
     </row>
     <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K393" s="1"/>
+      <c r="K393" s="5"/>
     </row>
     <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K394" s="1"/>
+      <c r="K394" s="5"/>
     </row>
     <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K395" s="1"/>
+      <c r="K395" s="5"/>
     </row>
     <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K396" s="1"/>
+      <c r="K396" s="5"/>
     </row>
     <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K397" s="1"/>
+      <c r="K397" s="5"/>
     </row>
     <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K398" s="1"/>
+      <c r="K398" s="5"/>
     </row>
     <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K399" s="1"/>
+      <c r="K399" s="5"/>
     </row>
     <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K400" s="1"/>
+      <c r="K400" s="5"/>
     </row>
     <row r="401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K401" s="1"/>
+      <c r="K401" s="5"/>
     </row>
     <row r="402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K402" s="1"/>
+      <c r="K402" s="5"/>
     </row>
     <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K403" s="1"/>
+      <c r="K403" s="5"/>
     </row>
     <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K404" s="1"/>
+      <c r="K404" s="5"/>
     </row>
     <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K405" s="1"/>
+      <c r="K405" s="5"/>
     </row>
     <row r="406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K406" s="1"/>
+      <c r="K406" s="5"/>
     </row>
     <row r="407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K407" s="1"/>
+      <c r="K407" s="5"/>
     </row>
     <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K408" s="1"/>
+      <c r="K408" s="5"/>
     </row>
     <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K409" s="1"/>
+      <c r="K409" s="5"/>
     </row>
     <row r="410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K410" s="1"/>
+      <c r="K410" s="5"/>
     </row>
     <row r="411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K411" s="1"/>
+      <c r="K411" s="5"/>
     </row>
     <row r="412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K412" s="1"/>
+      <c r="K412" s="5"/>
     </row>
     <row r="413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K413" s="1"/>
+      <c r="K413" s="5"/>
     </row>
     <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K414" s="1"/>
+      <c r="K414" s="5"/>
     </row>
     <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K415" s="1"/>
+      <c r="K415" s="5"/>
     </row>
     <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K416" s="1"/>
+      <c r="K416" s="5"/>
     </row>
     <row r="417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K417" s="1"/>
+      <c r="K417" s="5"/>
     </row>
     <row r="418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K418" s="1"/>
+      <c r="K418" s="5"/>
     </row>
     <row r="419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K419" s="1"/>
+      <c r="K419" s="5"/>
     </row>
     <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K420" s="1"/>
+      <c r="K420" s="5"/>
     </row>
     <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K421" s="1"/>
+      <c r="K421" s="5"/>
     </row>
     <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K422" s="1"/>
+      <c r="K422" s="5"/>
     </row>
     <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K423" s="1"/>
+      <c r="K423" s="5"/>
     </row>
     <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K424" s="1"/>
+      <c r="K424" s="5"/>
     </row>
     <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K425" s="1"/>
+      <c r="K425" s="5"/>
     </row>
     <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K426" s="1"/>
+      <c r="K426" s="5"/>
     </row>
     <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K427" s="1"/>
+      <c r="K427" s="5"/>
     </row>
     <row r="428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K428" s="1"/>
+      <c r="K428" s="5"/>
     </row>
     <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K429" s="1"/>
+      <c r="K429" s="5"/>
     </row>
     <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K430" s="1"/>
+      <c r="K430" s="5"/>
     </row>
     <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K431" s="1"/>
+      <c r="K431" s="5"/>
     </row>
     <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K432" s="1"/>
+      <c r="K432" s="5"/>
     </row>
     <row r="433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K433" s="1"/>
+      <c r="K433" s="5"/>
     </row>
     <row r="434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K434" s="1"/>
+      <c r="K434" s="5"/>
     </row>
     <row r="435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K435" s="1"/>
+      <c r="K435" s="5"/>
     </row>
     <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K436" s="1"/>
+      <c r="K436" s="5"/>
     </row>
     <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K437" s="1"/>
+      <c r="K437" s="5"/>
     </row>
     <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K438" s="1"/>
+      <c r="K438" s="5"/>
     </row>
     <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K439" s="1"/>
+      <c r="K439" s="5"/>
     </row>
     <row r="440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K440" s="1"/>
+      <c r="K440" s="5"/>
     </row>
     <row r="441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K441" s="1"/>
+      <c r="K441" s="5"/>
     </row>
     <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K442" s="1"/>
+      <c r="K442" s="5"/>
     </row>
     <row r="443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K443" s="1"/>
+      <c r="K443" s="5"/>
     </row>
     <row r="444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K444" s="1"/>
+      <c r="K444" s="5"/>
     </row>
     <row r="445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K445" s="1"/>
+      <c r="K445" s="5"/>
     </row>
     <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K446" s="1"/>
+      <c r="K446" s="5"/>
     </row>
     <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K447" s="1"/>
+      <c r="K447" s="5"/>
     </row>
     <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K448" s="1"/>
+      <c r="K448" s="5"/>
     </row>
     <row r="449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K449" s="1"/>
+      <c r="K449" s="5"/>
     </row>
     <row r="450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K450" s="1"/>
+      <c r="K450" s="5"/>
     </row>
     <row r="451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K451" s="1"/>
+      <c r="K451" s="5"/>
     </row>
     <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K452" s="1"/>
+      <c r="K452" s="5"/>
     </row>
     <row r="453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K453" s="1"/>
+      <c r="K453" s="5"/>
     </row>
     <row r="454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K454" s="1"/>
+      <c r="K454" s="5"/>
     </row>
     <row r="455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K455" s="1"/>
+      <c r="K455" s="5"/>
     </row>
     <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K456" s="1"/>
+      <c r="K456" s="5"/>
     </row>
     <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K457" s="1"/>
+      <c r="K457" s="5"/>
     </row>
     <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K458" s="1"/>
+      <c r="K458" s="5"/>
     </row>
     <row r="459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K459" s="1"/>
+      <c r="K459" s="5"/>
     </row>
     <row r="460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K460" s="1"/>
+      <c r="K460" s="5"/>
     </row>
     <row r="461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K461" s="1"/>
+      <c r="K461" s="5"/>
     </row>
     <row r="462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K462" s="1"/>
+      <c r="K462" s="5"/>
     </row>
     <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K463" s="1"/>
+      <c r="K463" s="5"/>
     </row>
     <row r="464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K464" s="1"/>
+      <c r="K464" s="5"/>
     </row>
     <row r="465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K465" s="1"/>
+      <c r="K465" s="5"/>
     </row>
     <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K466" s="1"/>
+      <c r="K466" s="5"/>
     </row>
     <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K467" s="1"/>
+      <c r="K467" s="5"/>
     </row>
     <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K468" s="1"/>
+      <c r="K468" s="5"/>
     </row>
     <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K469" s="1"/>
+      <c r="K469" s="5"/>
     </row>
     <row r="470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K470" s="1"/>
+      <c r="K470" s="5"/>
     </row>
     <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K471" s="1"/>
+      <c r="K471" s="5"/>
     </row>
     <row r="472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K472" s="1"/>
+      <c r="K472" s="5"/>
     </row>
     <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K473" s="1"/>
+      <c r="K473" s="5"/>
     </row>
     <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K474" s="1"/>
+      <c r="K474" s="5"/>
     </row>
     <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K475" s="1"/>
+      <c r="K475" s="5"/>
     </row>
     <row r="476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K476" s="1"/>
+      <c r="K476" s="5"/>
     </row>
     <row r="477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K477" s="1"/>
+      <c r="K477" s="5"/>
     </row>
     <row r="478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K478" s="1"/>
+      <c r="K478" s="5"/>
     </row>
     <row r="479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K479" s="1"/>
+      <c r="K479" s="5"/>
     </row>
     <row r="480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K480" s="1"/>
+      <c r="K480" s="5"/>
     </row>
     <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K481" s="1"/>
+      <c r="K481" s="5"/>
     </row>
     <row r="482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K482" s="1"/>
+      <c r="K482" s="5"/>
     </row>
     <row r="483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K483" s="1"/>
+      <c r="K483" s="5"/>
     </row>
     <row r="484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K484" s="1"/>
+      <c r="K484" s="5"/>
     </row>
     <row r="485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K485" s="1"/>
+      <c r="K485" s="5"/>
     </row>
     <row r="486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K486" s="1"/>
+      <c r="K486" s="5"/>
     </row>
     <row r="487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K487" s="1"/>
+      <c r="K487" s="5"/>
     </row>
     <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K488" s="1"/>
+      <c r="K488" s="5"/>
     </row>
     <row r="489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K489" s="1"/>
+      <c r="K489" s="5"/>
     </row>
     <row r="490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K490" s="1"/>
+      <c r="K490" s="5"/>
     </row>
     <row r="491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K491" s="1"/>
+      <c r="K491" s="5"/>
     </row>
     <row r="492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K492" s="1"/>
+      <c r="K492" s="5"/>
     </row>
     <row r="493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K493" s="1"/>
+      <c r="K493" s="5"/>
     </row>
     <row r="494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K494" s="1"/>
+      <c r="K494" s="5"/>
     </row>
     <row r="495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K495" s="1"/>
+      <c r="K495" s="5"/>
     </row>
     <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K496" s="1"/>
+      <c r="K496" s="5"/>
     </row>
     <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K497" s="1"/>
+      <c r="K497" s="5"/>
     </row>
     <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K498" s="1"/>
+      <c r="K498" s="5"/>
     </row>
     <row r="499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K499" s="1"/>
+      <c r="K499" s="5"/>
     </row>
     <row r="500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K500" s="1"/>
+      <c r="K500" s="5"/>
     </row>
     <row r="501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K501" s="1"/>
+      <c r="K501" s="5"/>
     </row>
     <row r="502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K502" s="1"/>
+      <c r="K502" s="5"/>
     </row>
     <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K503" s="1"/>
+      <c r="K503" s="5"/>
     </row>
     <row r="504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K504" s="1"/>
+      <c r="K504" s="5"/>
     </row>
     <row r="505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K505" s="1"/>
+      <c r="K505" s="5"/>
     </row>
     <row r="506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K506" s="1"/>
+      <c r="K506" s="5"/>
     </row>
     <row r="507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K507" s="1"/>
+      <c r="K507" s="5"/>
     </row>
     <row r="508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K508" s="1"/>
+      <c r="K508" s="5"/>
     </row>
     <row r="509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K509" s="1"/>
+      <c r="K509" s="5"/>
     </row>
     <row r="510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K510" s="1"/>
+      <c r="K510" s="5"/>
     </row>
     <row r="511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K511" s="1"/>
+      <c r="K511" s="5"/>
     </row>
     <row r="512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K512" s="1"/>
+      <c r="K512" s="5"/>
     </row>
     <row r="513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K513" s="1"/>
+      <c r="K513" s="5"/>
     </row>
     <row r="514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K514" s="1"/>
+      <c r="K514" s="5"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J500">
@@ -2024,7 +2557,7 @@
       <formula>"critical"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K514" type="list">
       <formula1>"not started,in progress,closed"</formula1>
       <formula2>0</formula2>
@@ -2037,8 +2570,12 @@
       <formula1>"Directed,Constrained Random,Random + Directed Stream,Error Injection,Reset/Init,Stress,Performance,Formal"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H55:H100" type="list">
       <formula1>"Code Coverage,Functional Coverage,Assertion,Formal Proof,Self-Checking Test"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H54" type="list">
+      <formula1>"Code Coverage,Functional Coverage,Assertion,Assertion + Coverage,Formal Proof,Self-Checking Test"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>